<commit_message>
Cleaning up redundancy in validation scenario names
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/Dehydration.xlsx
+++ b/data/human/adult/validation/Scenarios/Dehydration.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\dehydration\source\data\human\adult\validation\Scenarios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE50DB90-3996-4968-8050-00BCA8DDDD23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A720EC22-9E41-4BE2-9AED-BA50DCE0B0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29625" yWindow="8490" windowWidth="23130" windowHeight="19155" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6825" yWindow="3030" windowWidth="21600" windowHeight="12645" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="11" r:id="rId1"/>
-    <sheet name="MildDehydration" sheetId="7" r:id="rId2"/>
-    <sheet name="ModerateDehydration" sheetId="8" r:id="rId3"/>
-    <sheet name="SevereDehydration" sheetId="9" r:id="rId4"/>
+    <sheet name="Mild" sheetId="7" r:id="rId2"/>
+    <sheet name="Moderate" sheetId="8" r:id="rId3"/>
+    <sheet name="Severe" sheetId="9" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="39">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -146,15 +146,6 @@
               "Value": 0.5
             } } } }
 }</t>
-  </si>
-  <si>
-    <t>MildDehydration</t>
-  </si>
-  <si>
-    <t>ModerateDehydration</t>
-  </si>
-  <si>
-    <t>SevereDehydration</t>
   </si>
   <si>
     <t>Healthy standard male for comparison.</t>
@@ -314,25 +305,25 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -731,52 +722,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="24"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -788,11 +777,11 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -809,24 +798,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22" t="s">
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="22"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -835,22 +824,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="22"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -862,13 +851,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -876,13 +865,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -938,6 +927,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="G7:H7"/>
@@ -947,12 +942,6 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -980,52 +969,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="D2" s="24"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1037,13 +1024,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -1060,24 +1047,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22" t="s">
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="22"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1086,22 +1073,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="22"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1113,13 +1100,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -1127,13 +1114,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -1231,52 +1218,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="D2" s="24"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1288,13 +1273,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -1311,24 +1296,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22" t="s">
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="22"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1337,22 +1322,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="22"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1364,13 +1349,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -1378,13 +1363,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -1440,6 +1425,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B8:F8"/>
@@ -1450,11 +1440,6 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -1482,52 +1467,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="20"/>
+      <c r="D1" s="18"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="24"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="F2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1539,13 +1522,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -1562,24 +1545,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="20" t="s">
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="20"/>
+      <c r="H5" s="18"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22" t="s">
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="22"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1588,22 +1571,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="22"/>
+      <c r="H7" s="19"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1615,13 +1598,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -1629,13 +1612,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="B10" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -1691,6 +1674,11 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B8:F8"/>
@@ -1701,11 +1689,6 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Continued validatoin scenario renaming updates
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/Dehydration.xlsx
+++ b/data/human/adult/validation/Scenarios/Dehydration.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A720EC22-9E41-4BE2-9AED-BA50DCE0B0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C83850-1EF2-42B5-97C4-87B2F56E8F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6825" yWindow="3030" windowWidth="21600" windowHeight="12645" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -305,7 +305,16 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -315,15 +324,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -722,50 +722,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -777,11 +777,11 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -798,24 +798,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="19" t="s">
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -824,22 +824,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="19"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -851,13 +851,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -865,13 +865,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -927,12 +927,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="G7:H7"/>
@@ -942,6 +936,12 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -969,50 +969,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1024,13 +1024,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -1047,24 +1047,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="19" t="s">
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1073,22 +1073,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="19"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1100,13 +1100,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -1114,13 +1114,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -1218,50 +1218,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1273,13 +1273,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -1296,24 +1296,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="19" t="s">
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1322,22 +1322,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="19"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1349,13 +1349,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -1363,13 +1363,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -1425,11 +1425,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B8:F8"/>
@@ -1440,6 +1435,11 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -1467,50 +1467,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="18"/>
+      <c r="D1" s="20"/>
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" ht="129" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
       <c r="E2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
       <c r="G3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1522,13 +1522,13 @@
       <c r="A4" s="10">
         <v>0</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="4"/>
       <c r="H4" s="17"/>
     </row>
@@ -1545,24 +1545,24 @@
       <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="18" t="s">
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="18"/>
+      <c r="H5" s="20"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="10"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="19" t="s">
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
@@ -1571,22 +1571,22 @@
       <c r="D7" s="10"/>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="19"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="1" t="s">
         <v>7</v>
       </c>
@@ -1598,13 +1598,13 @@
       <c r="A9" s="12">
         <v>1</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
       <c r="G9" s="13"/>
       <c r="H9" s="17"/>
     </row>
@@ -1612,13 +1612,13 @@
       <c r="A10" s="10">
         <v>1</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
       <c r="G10" s="4"/>
       <c r="H10" s="17" t="s">
         <v>32</v>
@@ -1674,11 +1674,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B8:F8"/>
@@ -1689,6 +1684,11 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F6"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>